<commit_message>
Minor definition wording change.
</commit_message>
<xml_diff>
--- a/data/source/codebook.xlsx
+++ b/data/source/codebook.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/leopallen/Documents/research/wikipedia_discourse/codebooks/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/leopallen/Documents/research/wikipedia_discourse/human_annotation_tool/data/source/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{99B380A4-1C6B-9B40-A65D-6E735B27811B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{815EB74C-A7EB-D74C-9491-EFC6B072BE19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17240" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Core_Schema" sheetId="1" r:id="rId1"/>
@@ -217,9 +217,6 @@
 https://aclanthology.org/2024.nlpcss-1.1/</t>
   </si>
   <si>
-    <t>The utterance states or challenges a position about the article or the dispute.</t>
-  </si>
-  <si>
     <t>The utterance takes a position that makes a clear claim about a specific clear target issue</t>
   </si>
   <si>
@@ -653,6 +650,9 @@
   </si>
   <si>
     <t>If KI_present=1, code 1 when the speaker reports a completed or initiated edit/action and frames it as responsive to the dispute. Code 0 for proposals, another person’s edit used only as evidence, or a bare adversarial revert not presented as a candidate route to resolution. If KI_present=0, return null.</t>
+  </si>
+  <si>
+    <t>The utterance states or challenges a personal position about the article or the dispute.</t>
   </si>
 </sst>
 </file>
@@ -976,10 +976,10 @@
         <v>9</v>
       </c>
       <c r="D2" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>194</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>195</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>10</v>
@@ -999,10 +999,10 @@
         <v>9</v>
       </c>
       <c r="D3" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>196</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>197</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>13</v>
@@ -1022,10 +1022,10 @@
         <v>9</v>
       </c>
       <c r="D4" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>198</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>199</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>15</v>
@@ -1042,13 +1042,13 @@
         <v>16</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>17</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>18</v>
@@ -1065,13 +1065,13 @@
         <v>19</v>
       </c>
       <c r="C6" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="D6" s="1" t="s">
-        <v>158</v>
-      </c>
       <c r="E6" s="1" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="F6" s="3" t="s">
         <v>20</v>
@@ -1094,7 +1094,7 @@
         <v>22</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>23</v>
@@ -1114,10 +1114,10 @@
         <v>9</v>
       </c>
       <c r="D8" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="E8" s="1" t="s">
         <v>160</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>161</v>
       </c>
       <c r="F8" s="3" t="s">
         <v>25</v>
@@ -1140,7 +1140,7 @@
         <v>27</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>28</v>
@@ -1160,10 +1160,10 @@
         <v>9</v>
       </c>
       <c r="D10" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="E10" s="1" t="s">
         <v>200</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>201</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>31</v>
@@ -1183,10 +1183,10 @@
         <v>9</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>33</v>
@@ -1206,10 +1206,10 @@
         <v>9</v>
       </c>
       <c r="D12" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="E12" s="1" t="s">
         <v>203</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>204</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>35</v>
@@ -1232,7 +1232,7 @@
         <v>37</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>38</v>
@@ -1255,7 +1255,7 @@
         <v>40</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>38</v>
@@ -1272,16 +1272,16 @@
         <v>41</v>
       </c>
       <c r="C15" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="D15" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="D15" s="1" t="s">
+      <c r="E15" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="F15" s="2" t="s">
         <v>167</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>187</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>168</v>
       </c>
       <c r="G15" s="1" t="s">
         <v>11</v>
@@ -1295,16 +1295,16 @@
         <v>42</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D16" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="F16" s="3" t="s">
         <v>169</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>188</v>
-      </c>
-      <c r="F16" s="3" t="s">
-        <v>170</v>
       </c>
       <c r="G16" s="1" t="s">
         <v>11</v>
@@ -1435,10 +1435,10 @@
         <v>9</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>59</v>
+        <v>204</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>10</v>
@@ -1458,10 +1458,10 @@
         <v>9</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>13</v>
@@ -1481,10 +1481,10 @@
         <v>9</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>15</v>
@@ -1501,13 +1501,13 @@
         <v>16</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>18</v>
@@ -1524,13 +1524,13 @@
         <v>19</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>20</v>
@@ -1550,10 +1550,10 @@
         <v>9</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>23</v>
@@ -1573,10 +1573,10 @@
         <v>9</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>25</v>
@@ -1596,10 +1596,10 @@
         <v>9</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>28</v>
@@ -1619,10 +1619,10 @@
         <v>9</v>
       </c>
       <c r="D10" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E10" s="1" t="s">
         <v>66</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>67</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>31</v>
@@ -1642,10 +1642,10 @@
         <v>9</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="F11" s="1" t="s">
         <v>33</v>
@@ -1665,10 +1665,10 @@
         <v>9</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F12" s="1" t="s">
         <v>35</v>
@@ -1688,10 +1688,10 @@
         <v>9</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F13" s="1" t="s">
         <v>38</v>
@@ -1711,10 +1711,10 @@
         <v>9</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="F14" s="1" t="s">
         <v>38</v>
@@ -1731,16 +1731,16 @@
         <v>41</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D15" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="E15" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="E15" s="1" t="s">
-        <v>184</v>
-      </c>
       <c r="F15" s="1" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G15" s="1" t="s">
         <v>11</v>
@@ -1754,16 +1754,16 @@
         <v>42</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E16" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="F16" s="1" t="s">
         <v>190</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>191</v>
       </c>
       <c r="G16" s="1" t="s">
         <v>11</v>
@@ -1780,10 +1780,10 @@
         <v>9</v>
       </c>
       <c r="D17" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E17" s="1" t="s">
         <v>72</v>
-      </c>
-      <c r="E17" s="1" t="s">
-        <v>73</v>
       </c>
       <c r="F17" s="1" t="s">
         <v>47</v>
@@ -1803,10 +1803,10 @@
         <v>9</v>
       </c>
       <c r="D18" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="E18" s="1" t="s">
         <v>74</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>75</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>51</v>
@@ -1826,13 +1826,13 @@
         <v>54</v>
       </c>
       <c r="D19" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="E19" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="E19" s="1" t="s">
-        <v>77</v>
-      </c>
       <c r="F19" s="1" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="G19" s="1"/>
     </row>
@@ -1859,39 +1859,39 @@
   <sheetData>
     <row r="1" spans="1:6" ht="50" customHeight="1">
       <c r="A1" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>3</v>
       </c>
       <c r="C1" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="D1" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="E1" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>81</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="80" customHeight="1">
       <c r="A2" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="C2" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="D2" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" s="3" t="s">
         <v>86</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>87</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>11</v>
@@ -1899,19 +1899,19 @@
     </row>
     <row r="3" spans="1:6" ht="72" customHeight="1">
       <c r="A3" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="E3" s="3" t="s">
         <v>91</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>92</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>11</v>
@@ -1919,19 +1919,19 @@
     </row>
     <row r="4" spans="1:6" ht="112" customHeight="1">
       <c r="A4" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="C4" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="D4" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="E4" s="3" t="s">
         <v>96</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>97</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>11</v>
@@ -1939,19 +1939,19 @@
     </row>
     <row r="5" spans="1:6" ht="96" customHeight="1">
       <c r="A5" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="C5" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="D5" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="E5" s="3" t="s">
         <v>101</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>102</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>11</v>
@@ -1959,19 +1959,19 @@
     </row>
     <row r="6" spans="1:6" ht="112" customHeight="1">
       <c r="A6" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="C6" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="D6" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="E6" s="3" t="s">
         <v>106</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>107</v>
       </c>
       <c r="F6" s="3" t="s">
         <v>11</v>
@@ -1979,19 +1979,19 @@
     </row>
     <row r="7" spans="1:6" ht="96" customHeight="1">
       <c r="A7" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="C7" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="D7" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="E7" s="3" t="s">
         <v>111</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>112</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>11</v>
@@ -1999,19 +1999,19 @@
     </row>
     <row r="8" spans="1:6" ht="96" customHeight="1">
       <c r="A8" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="C8" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="D8" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="E8" s="3" t="s">
         <v>116</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>117</v>
       </c>
       <c r="F8" s="3" t="s">
         <v>11</v>
@@ -2039,33 +2039,33 @@
   <sheetData>
     <row r="1" spans="1:5" ht="50" customHeight="1">
       <c r="A1" s="4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>3</v>
       </c>
       <c r="C1" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="D1" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="D1" s="4" t="s">
-        <v>120</v>
-      </c>
       <c r="E1" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="96" customHeight="1">
       <c r="A2" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>123</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>124</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>11</v>
@@ -2073,16 +2073,16 @@
     </row>
     <row r="3" spans="1:5" ht="96" customHeight="1">
       <c r="A3" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="C3" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="D3" s="1" t="s">
         <v>127</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>128</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>11</v>
@@ -2090,16 +2090,16 @@
     </row>
     <row r="4" spans="1:5" ht="96" customHeight="1">
       <c r="A4" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="C4" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="D4" s="1" t="s">
         <v>131</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>132</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>11</v>
@@ -2107,16 +2107,16 @@
     </row>
     <row r="5" spans="1:5" ht="96" customHeight="1">
       <c r="A5" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="C5" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="D5" s="1" t="s">
         <v>135</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>136</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>11</v>
@@ -2124,16 +2124,16 @@
     </row>
     <row r="6" spans="1:5" ht="96" customHeight="1">
       <c r="A6" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="C6" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="D6" s="1" t="s">
         <v>139</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>140</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>11</v>
@@ -2141,16 +2141,16 @@
     </row>
     <row r="7" spans="1:5" ht="96" customHeight="1">
       <c r="A7" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="C7" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="D7" s="1" t="s">
         <v>143</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>144</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>11</v>
@@ -2158,16 +2158,16 @@
     </row>
     <row r="8" spans="1:5" ht="96" customHeight="1">
       <c r="A8" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="C8" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="D8" s="1" t="s">
         <v>147</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>148</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>11</v>
@@ -2175,16 +2175,16 @@
     </row>
     <row r="9" spans="1:5" ht="96" customHeight="1">
       <c r="A9" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="D9" s="1" t="s">
         <v>151</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>152</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>11</v>
@@ -2192,13 +2192,13 @@
     </row>
     <row r="10" spans="1:5" ht="96" customHeight="1">
       <c r="A10" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="B10" s="1" t="s">
-        <v>154</v>
-      </c>
       <c r="C10" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D10" s="1"/>
       <c r="E10" s="1" t="s">

</xml_diff>

<commit_message>
RElaxing the KS, KI evidence fields to optional for human annotation.
</commit_message>
<xml_diff>
--- a/data/source/codebook.xlsx
+++ b/data/source/codebook.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/leopallen/Documents/research/wikipedia_discourse/human_annotation_tool/data/source/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{815EB74C-A7EB-D74C-9491-EFC6B072BE19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13DBC9B5-8C48-FA4C-B06B-0BF7A12309B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17240" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Core_Schema" sheetId="1" r:id="rId1"/>
@@ -508,9 +508,6 @@
     <t>Only code this field when KS_evidence_present=1. Assign every applicable label from Evidence_Types, using each label at most once. Do not force one primary type. If KS_evidence_present=0 or null, return null.</t>
   </si>
   <si>
-    <t>binary option {0,1}; ordinal option {1,2,3,4,5}; null when not applicable</t>
-  </si>
-  <si>
     <t>A warrant is the stated reasoning or rule that explains how the identified evidence supports the claim. This construct may be recorded either as binary warrant presence or as the degree to which the warrant is explicit and clear.</t>
   </si>
   <si>
@@ -595,21 +592,9 @@
     <t>Prior-stake reflection captures how much a candidate action appears to reuse substantive knowledge staked earlier in the dispute. The contributor does not need to mention or acknowledge the earlier stake.</t>
   </si>
   <si>
-    <t xml:space="preserve">Apply only when KS_present=1 and KS_evidence_present=1; otherwise return null. BINARY OPTION: 1 = the utterance states a warrant linking the evidence to the claim; 0 = no warrant is stated and the link must be inferred. ORDINAL OPTION: rate agreement with ‘The warrant explaining how the identified evidence supports the claim is explicit and clear.’ 1 = strongly disagree, no warrant is stated; 2 = disagree, only a vague or ambiguous link is stated; 3 = neither agree nor disagree, a discernible link is stated, but it is incomplete or unclear; 4 = agree, the link is explicit and mostly clear; 5 = strongly agree, the link is explicit, clear, and specific. </t>
-  </si>
-  <si>
     <t>Assign one label only when the utterance explicitly evaluates an earlier candidate action. accept = explicitly accepts the candidate or a substantive part or direction without also rejecting or conditioning it. reject = explicitly rejects the candidate and accepts no substantive part or direction. mixed_or_conditional = explicitly accepts some part only under stated conditions, or accepts one part while rejecting or qualifying another. When there is no explicit evaluation, leave null. This includes cases with KI_present=0 or no earlier candidate action.</t>
   </si>
   <si>
-    <t>Apply only when KI_present=1 and at least one earlier utterance has KS_present=1; otherwise return null. BINARY OPTION: 1 = the candidate action appears to reuse or incorporate an identifiable substantive element or constraint from at least one earlier stake; 0 = no identifiable reuse or incorporation. ORDINAL OPTION: rate agreement with ‘The candidate action incorporates substantive knowledge staked earlier in the dispute.’ 1 = strongly disagree, no identifiable reuse; 2 = disagree, only slight or tenuous reuse of a peripheral element; 3 = neither agree nor disagree, discernible but partial reuse of a substantive element; 4 = agree, substantial incorporation of the content or constraint of at least one earlier stake; 5 = strongly agree, extensive incorporation or recombination such that earlier staked knowledge materially impacts the candidate edit/action. Infer from correspondence between the candidate action’s content and earlier staked knoweldge in the dialogue.</t>
-  </si>
-  <si>
-    <t>Use only when KS_present=1 and KS_evidence_present=1; otherwise return null. BINARY OPTION: 1 = a warrant linking evidence to claim is stated; 0 = the link must be inferred. ORDINAL OPTION: rate ‘The warrant explaining how the evidence supports the claim is explicit and clear.’ 1 = strongly disagree: no warrant; 2 = disagree: vague or ambiguous link; 3 = neither agree nor disagree: a partial or unclear link; 4 = agree: an explicit and mostly clear link; 5 = strongly agree: an explicit, clear, and specific link.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Use only when KI_present=1 and at least one earlier KS utterance exists; otherwise return null. BINARY OPTION: 1 = the candidate appears to reuse or incorporate an identifiable substantive element or constraint from an earlier stake; 0 = no identifiable reuse. ORDINAL OPTION: rate ‘The candidate action incorporates substantive knowledge staked earlier in the dispute.’ 1 = strongly disagree: no identifiable reuse; 2 = disagree: slight or tenuous reuse of a peripheral element; 3 = neither agree nor disagree: discernible but partial reuse of a substantive element; 4 = agree: substantial incorporation of an earlier stake’s content or constraint; 5 = strongly agree: extensive incorporation or recombination that materially structures the candidate action. Judge reuse from the candidate’s content and the earlier dialogue. </t>
-  </si>
-  <si>
     <t>[WikiTactics | conv_id=253990014.204845.204845 | utterance_index=7; reflects utterance_indices=0,3,4,6] “call it ‘Civilians’ or ‘Civilians and non-combatants’” implicitly reuses the earlier distinction between narrow legal and broader dictionary meanings of “non-combatant,” (without explicitly acknowledging earlier staked knowledge).</t>
   </si>
   <si>
@@ -653,6 +638,21 @@
   </si>
   <si>
     <t>The utterance states or challenges a personal position about the article or the dispute.</t>
+  </si>
+  <si>
+    <t>Use only when KS_present=1 and KS_evidence_present=1; otherwise return null. Rate ‘The warrant explaining how the evidence supports the claim is explicit and clear.’ 1 = strongly disagree: no warrant; 2 = disagree: vague or ambiguous link; 3 = neither agree nor disagree: a partial or unclear link; 4 = agree: an explicit and mostly clear link; 5 = strongly agree: an explicit, clear, and specific link.</t>
+  </si>
+  <si>
+    <t>ordinal {1,2,3,4,5}; null when not applicable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Use only when KI_present=1 and at least one earlier KS utterance exists; otherwise return null. Rate ‘The candidate action incorporates substantive knowledge staked earlier in the dispute.’ 1 = strongly disagree: no identifiable reuse; 2 = disagree: slight or tenuous reuse of a peripheral element; 3 = neither agree nor disagree: discernible but partial reuse of a substantive element; 4 = agree: substantial incorporation of an earlier stake’s content or constraint; 5 = strongly agree: extensive incorporation or recombination that materially structures the candidate action. Judge reuse from the candidate’s content and the earlier dialogue. </t>
+  </si>
+  <si>
+    <t>Apply only when KI_present=1 and at least one earlier utterance has KS_present=1; otherwise return null. Rate agreement with ‘The candidate action incorporates substantive knowledge staked earlier in the dispute.’ 1 = strongly disagree, no identifiable reuse; 2 = disagree, only slight or tenuous reuse of a peripheral element; 3 = neither agree nor disagree, discernible but partial reuse of a substantive element; 4 = agree, substantial incorporation of the content or constraint of at least one earlier stake; 5 = strongly agree, extensive incorporation or recombination such that earlier staked knowledge materially impacts the candidate edit/action. Infer from correspondence between the candidate action’s content and earlier staked knoweldge in the dialogue.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apply only when KS_present=1 and KS_evidence_present=1; otherwise return null. Rate agreement with ‘The warrant explaining how the identified evidence supports the claim is explicit and clear.’ 1 = strongly disagree, no warrant is stated; 2 = disagree, only a vague or ambiguous link is stated; 3 = neither agree nor disagree, a discernible link is stated, but it is incomplete or unclear; 4 = agree, the link is explicit and mostly clear; 5 = strongly agree, the link is explicit, clear, and specific. </t>
   </si>
 </sst>
 </file>
@@ -931,7 +931,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
@@ -976,10 +976,10 @@
         <v>9</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>10</v>
@@ -999,10 +999,10 @@
         <v>9</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>13</v>
@@ -1022,10 +1022,10 @@
         <v>9</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>15</v>
@@ -1065,13 +1065,13 @@
         <v>19</v>
       </c>
       <c r="C6" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="D6" s="1" t="s">
-        <v>157</v>
-      </c>
       <c r="E6" s="1" t="s">
-        <v>185</v>
+        <v>204</v>
       </c>
       <c r="F6" s="3" t="s">
         <v>20</v>
@@ -1094,7 +1094,7 @@
         <v>22</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>23</v>
@@ -1114,10 +1114,10 @@
         <v>9</v>
       </c>
       <c r="D8" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="E8" s="1" t="s">
         <v>159</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>160</v>
       </c>
       <c r="F8" s="3" t="s">
         <v>25</v>
@@ -1140,7 +1140,7 @@
         <v>27</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>28</v>
@@ -1160,10 +1160,10 @@
         <v>9</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>31</v>
@@ -1183,10 +1183,10 @@
         <v>9</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>33</v>
@@ -1206,10 +1206,10 @@
         <v>9</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>35</v>
@@ -1232,7 +1232,7 @@
         <v>37</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>38</v>
@@ -1255,7 +1255,7 @@
         <v>40</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>38</v>
@@ -1272,16 +1272,16 @@
         <v>41</v>
       </c>
       <c r="C15" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="D15" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="D15" s="1" t="s">
+      <c r="E15" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="F15" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="G15" s="1" t="s">
         <v>11</v>
@@ -1295,16 +1295,16 @@
         <v>42</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>156</v>
+        <v>201</v>
       </c>
       <c r="D16" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="F16" s="3" t="s">
         <v>168</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>187</v>
-      </c>
-      <c r="F16" s="3" t="s">
-        <v>169</v>
       </c>
       <c r="G16" s="1" t="s">
         <v>11</v>
@@ -1390,7 +1390,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
@@ -1435,10 +1435,10 @@
         <v>9</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>10</v>
@@ -1461,7 +1461,7 @@
         <v>59</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>13</v>
@@ -1484,7 +1484,7 @@
         <v>60</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>15</v>
@@ -1507,7 +1507,7 @@
         <v>61</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>18</v>
@@ -1524,13 +1524,13 @@
         <v>19</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>156</v>
+        <v>201</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>188</v>
+        <v>200</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>20</v>
@@ -1553,7 +1553,7 @@
         <v>62</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>23</v>
@@ -1576,7 +1576,7 @@
         <v>63</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>25</v>
@@ -1599,7 +1599,7 @@
         <v>64</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>28</v>
@@ -1645,7 +1645,7 @@
         <v>67</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F11" s="1" t="s">
         <v>33</v>
@@ -1668,7 +1668,7 @@
         <v>68</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="F12" s="1" t="s">
         <v>35</v>
@@ -1691,7 +1691,7 @@
         <v>69</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F13" s="1" t="s">
         <v>38</v>
@@ -1714,7 +1714,7 @@
         <v>70</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F14" s="1" t="s">
         <v>38</v>
@@ -1731,16 +1731,16 @@
         <v>41</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D15" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="E15" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="E15" s="1" t="s">
-        <v>183</v>
-      </c>
       <c r="F15" s="1" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="G15" s="1" t="s">
         <v>11</v>
@@ -1754,16 +1754,16 @@
         <v>42</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>156</v>
+        <v>201</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>189</v>
+        <v>202</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="G16" s="1" t="s">
         <v>11</v>
@@ -1832,7 +1832,7 @@
         <v>76</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="G19" s="1"/>
     </row>
@@ -1847,7 +1847,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:F8"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
     <col min="2" max="2" width="54" customWidth="1"/>
@@ -2028,7 +2028,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
     <col min="2" max="2" width="55" customWidth="1"/>
@@ -2198,7 +2198,7 @@
         <v>153</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="D10" s="1"/>
       <c r="E10" s="1" t="s">

</xml_diff>

<commit_message>
Pushing post-meeting changes to schema and annotation UI
</commit_message>
<xml_diff>
--- a/data/source/codebook.xlsx
+++ b/data/source/codebook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/leopallen/Documents/research/wikipedia_discourse/human_annotation_tool/data/source/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B96AD73-53A3-9A4F-A36F-89C5417868B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A04108B-528F-5340-BCDE-1C8A174E4A0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="214">
   <si>
     <t>Family</t>
   </si>
@@ -142,9 +142,6 @@
     <t>binary {0,1}; null unless KS_present=1 and an earlier KS exists</t>
   </si>
   <si>
-    <t>Whether the utterance repeats substantive knowledge already present in the dispute without materially improving the pool of staked knowledge.</t>
-  </si>
-  <si>
     <t>Raw text: “We have many different reliable sources each stating different dates. Do you see the issue?”
 Explanation: The same reliable-sources/different-dates point was already present earlier in the dispute, and this utterance adds no evidence, reasoning, qualification, or implication.</t>
   </si>
@@ -159,12 +156,6 @@
     <t>KI_present</t>
   </si>
   <si>
-    <t>Whether the utterance engages an identifiable candidate article edit by proposing it, reporting its implementation, revising it, soliciting feedback on it, or evaluating it.</t>
-  </si>
-  <si>
-    <t>Code 1 when the utterance engages a candidate article edit. Explicit rejection of an earlier candidate counts. Code 0 for a pure article-level claim or objection with no candidate edit, and for a generic process or governance step. KS and KI may co-occur.</t>
-  </si>
-  <si>
     <t>Raw text: “Okay, well how about we call it ‘Civilians’ or ‘Civilians and non-combatants’ instead?”
 Explanation: The utterance engages a concrete candidate article edit.</t>
   </si>
@@ -210,9 +201,6 @@
   </si>
   <si>
     <t>binary {0,1}; null unless KI_present=1 and an earlier candidate exists</t>
-  </si>
-  <si>
-    <t>Whether the utterance materially modifies, combines, narrows, extends, implements, or repairs an identifiable earlier candidate edit.</t>
   </si>
   <si>
     <t>Raw text: “OK, I cut the text down from one of the pictures, and ‘hid’ some of the text for another. Is this any better?”
@@ -246,9 +234,6 @@
     <t>binary {0,1}; null unless KI_present=1 and an earlier KS exists</t>
   </si>
   <si>
-    <t>Whether the candidate edit or its evaluation visibly reuses knowledge staked earlier in the dispute.</t>
-  </si>
-  <si>
     <t>Raw text: “I’ve moved the element of critical evaluation into the Critical reaction section per your observation.”
 Explanation: “Per your observation” identifies earlier staked knowledge and states how it shaped the enacted edit.</t>
   </si>
@@ -612,15 +597,6 @@
   </si>
   <si>
     <t>Only code if KI_present=1; otherwise null. Code 1 when the contributor says they already changed, added, removed, moved, restored, sourced, tagged, or otherwise edited the article and frames that edit as responsive to the dispute. A bare adversarial revert is 0 unless presented as a solution.</t>
-  </si>
-  <si>
-    <t>Only code if KI_present=1; otherwise null. Code 1 when the utterance explicitly asks for feedback, objections, agreement, review, or further revision of a visible candidate edit. A generic “comments?” with no candidate and a request for facts unrelated to a candidate are 0.</t>
-  </si>
-  <si>
-    <t>Only code if KI_present=1 and an earlier utterance has KI_present=1 and identifies the candidate being revised; otherwise null. Code 1 when that earlier candidate is used as a baseline and substantively changed. Verbatim repetition, acknowledgment, acceptance, rejection, or introduction of an unrelated new edit is 0.</t>
-  </si>
-  <si>
-    <t>Only code if KI_present=1 and an earlier utterance has KI_present=1 and identifies the candidate being evaluated; otherwise null. Assign one label only. accept = accepts the candidate or a substantive part without rejection or condition. reject = rejects it and accepts no substantive part. mixed_or_conditional = accepts only under a condition or accepts one part while rejecting or qualifying another.</t>
   </si>
   <si>
     <t>Only code if KI_present=1 and at least one earlier utterance has KS_present=1; otherwise null. Code 1 only when the coder can identify an earlier claim, objection, reasoning, evidence item, or constraint from a prior KS utterance that shapes the focal utterance. Mere acknowledgment, topical overlap, or a speculative connection is 0. Do not rate depth or quality.</t>
@@ -688,6 +664,69 @@
   </si>
   <si>
     <t>How convincingly the evidence and reasoning offered, taken as a whole, support the specified claim(s) as stated. This is a bounded global judgment of the argument-claim relationship, deliberately combining relevance, completeness, consistency, and convincingness while excluding source-status and style judgments.</t>
+  </si>
+  <si>
+    <t>KS_warrant_reasoning</t>
+  </si>
+  <si>
+    <t>Whether the utterance develops a logical line of reasoning that connects supporting evidence, or a premise, to a conclusion or claim.</t>
+  </si>
+  <si>
+    <t>Only code if KS_present=1; otherwise null. Code 1 when the utterance develops an explicit line of reasoning that connects supporting evidence or a stated premise to a conclusion or claim. Code 0 when the utterance merely states a premise, names or quotes evidence, or asserts a conclusion without explaining how the premise or evidence supports it. KS_warrant_reasoning and KS_evidence_present may both be 1.</t>
+  </si>
+  <si>
+    <t>Whether the utterance repeats substantive knowledge already present in the dispute without materially developing the pool of staked knowledge.</t>
+  </si>
+  <si>
+    <t>Whether the utterance engages an identifiable article edit by proposing it, reporting its implementation, revising it, soliciting feedback on it, or evaluating it.</t>
+  </si>
+  <si>
+    <t>Whether the contributor reports implementing an edit as a proposed solution or trial.</t>
+  </si>
+  <si>
+    <t>Only code if KI_present=1 and an earlier utterance has KI_present=1 and identifies/describes/references an edit that could be revised; otherwise null. Code 1 when that earlier edit is used as a starting point and that the focal utterance somehow develops. Verbatim repetition, acknowledgment, acceptance, rejection, or introduction of an unrelated new edit is 0.</t>
+  </si>
+  <si>
+    <t>Code 1 when the utterance engages (i.e., assesses, proposes, makes, refines) an article edit. Explicit rejection of an earlier proposal counts. Code 0 for a pure article-level claim or objection with no proposed edit, and for a generic process or governance step. Code 0 for utterances that call for unelaborated reverts of another contributor's work. KS and KI may co-occur.</t>
+  </si>
+  <si>
+    <t>Raw text: “Okay, well how about we call it ‘Civilians’ or ‘Civilians and non-combatants’ instead?”
+Explanation: The utterance proposes two concrete article edits.</t>
+  </si>
+  <si>
+    <t>KI_solicit_feedback</t>
+  </si>
+  <si>
+    <t>Only code if KI_present=1; otherwise null. Code 1 when the utterance explicitly asks for feedback, objections, agreement, review, or further revision of a possible resolution (e.g., a proposed edit). A generic “comments?” with no proposed or enacted edit, and a request for facts unrelated to a proposed/enacted edit are 0.</t>
+  </si>
+  <si>
+    <t>Whether the contributor explicitly accepts, rejects, or gives a mixed or conditional evaluation of an earlier proposed edit.</t>
+  </si>
+  <si>
+    <t>Whether the edit or its evaluation visibly reuses knowledge staked earlier in the dispute.</t>
+  </si>
+  <si>
+    <t>KI_iterate</t>
+  </si>
+  <si>
+    <t>Whether the utterance materially modifies, combines, narrows, extends, implements, or repairs an identifiable an edit proposed/enacted earlier.</t>
+  </si>
+  <si>
+    <t>Only code if KI_present=1 and an earlier utterance has KI_present=1; otherwise null. Assign one label only. accept = accepts the edit or a substantive part without rejection or condition. reject = rejects it and accepts no substantive part. mixed_or_conditional = accepts only under a condition or accepts one part while rejecting or qualifying another.</t>
+  </si>
+  <si>
+    <t>Accept — Raw text: “your fourth source seems ok to me… Feel free to add the content.”
+Explanation: The contributor explicitly authorizes the addition.
+Reject — Raw text: “Just adding pictures… is a solution which has previously been discussed and rejected…”
+Explanation: The edit is explicitly rejected.
+Mixed/conditional — Raw text: “I’m fine with tweaking section headers, but…”
+Explanation: One part is accepted while the broader edit is qualified or opposed.</t>
+  </si>
+  <si>
+    <t>binary {0,1}; null unless KI_present=1 and an earlier KI attempt exists</t>
+  </si>
+  <si>
+    <t>Whether the contributor asks others to assess, revise, or accept, their work.</t>
   </si>
 </sst>
 </file>
@@ -984,10 +1023,10 @@
         <v>15</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>16</v>
@@ -1010,7 +1049,7 @@
         <v>19</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>20</v>
@@ -1033,7 +1072,7 @@
         <v>23</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>24</v>
@@ -1047,22 +1086,22 @@
         <v>7</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>26</v>
+        <v>195</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>200</v>
+        <v>192</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="258" customHeight="1">
@@ -1079,7 +1118,7 @@
         <v>29</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>30</v>
@@ -1099,36 +1138,36 @@
         <v>33</v>
       </c>
       <c r="D8" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="F8" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="E8" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="F8" s="1" t="s">
+      <c r="G8" s="1" t="s">
         <v>35</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="117.25" customHeight="1">
       <c r="A9" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>37</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>38</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>9</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>39</v>
+        <v>199</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>40</v>
+        <v>202</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>41</v>
+        <v>203</v>
       </c>
       <c r="G9" s="1" t="s">
         <v>17</v>
@@ -1136,22 +1175,22 @@
     </row>
     <row r="10" spans="1:7" ht="117.25" customHeight="1">
       <c r="A10" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B10" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="F10" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>45</v>
       </c>
       <c r="G10" s="1" t="s">
         <v>17</v>
@@ -1159,22 +1198,22 @@
     </row>
     <row r="11" spans="1:7" ht="117.25" customHeight="1">
       <c r="A11" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>47</v>
+        <v>200</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="G11" s="1" t="s">
         <v>13</v>
@@ -1182,91 +1221,91 @@
     </row>
     <row r="12" spans="1:7" ht="117.25" customHeight="1">
       <c r="A12" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B12" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="G12" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="G12" s="1" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="117.25" customHeight="1">
       <c r="A13" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>53</v>
+        <v>208</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>54</v>
+        <v>212</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>55</v>
+        <v>209</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>180</v>
+        <v>201</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="164.25" customHeight="1">
       <c r="A14" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B14" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="G14" s="1" t="s">
         <v>57</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="117.25" customHeight="1">
       <c r="A15" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>64</v>
+        <v>207</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>182</v>
+        <v>174</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="G15" s="1" t="s">
         <v>13</v>
@@ -1274,91 +1313,91 @@
     </row>
     <row r="16" spans="1:7" ht="117.25" customHeight="1">
       <c r="A16" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>9</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="117.25" customHeight="1">
       <c r="A17" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>9</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="117.25" customHeight="1">
       <c r="A18" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>9</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="117.25" customHeight="1">
       <c r="A19" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="F19" s="1" t="s">
         <v>81</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="E19" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>86</v>
       </c>
       <c r="G19" s="1" t="s">
         <v>13</v>
@@ -1416,10 +1455,10 @@
         <v>9</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>12</v>
@@ -1439,10 +1478,10 @@
         <v>15</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>183</v>
+        <v>175</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>16</v>
@@ -1462,10 +1501,10 @@
         <v>15</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>20</v>
@@ -1485,10 +1524,10 @@
         <v>22</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>185</v>
+        <v>177</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>24</v>
@@ -1508,16 +1547,16 @@
         <v>15</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>200</v>
+        <v>192</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="193.5" customHeight="1">
@@ -1531,10 +1570,10 @@
         <v>28</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>30</v>
@@ -1554,36 +1593,36 @@
         <v>33</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="F8" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="G8" s="1" t="s">
         <v>35</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="88" customHeight="1">
       <c r="A9" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>37</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>38</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>9</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="G9" s="1" t="s">
         <v>17</v>
@@ -1591,22 +1630,22 @@
     </row>
     <row r="10" spans="1:7" ht="88" customHeight="1">
       <c r="A10" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B10" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="F10" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>188</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>45</v>
       </c>
       <c r="G10" s="1" t="s">
         <v>17</v>
@@ -1614,22 +1653,22 @@
     </row>
     <row r="11" spans="1:7" ht="88" customHeight="1">
       <c r="A11" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="G11" s="1" t="s">
         <v>13</v>
@@ -1637,91 +1676,91 @@
     </row>
     <row r="12" spans="1:7" ht="88" customHeight="1">
       <c r="A12" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B12" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="G12" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>190</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="G12" s="1" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="88" customHeight="1">
       <c r="A13" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="123.25" customHeight="1">
       <c r="A14" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B14" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="G14" s="1" t="s">
         <v>57</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>192</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="88" customHeight="1">
       <c r="A15" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>193</v>
+        <v>185</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>194</v>
+        <v>186</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="G15" s="1" t="s">
         <v>13</v>
@@ -1729,91 +1768,91 @@
     </row>
     <row r="16" spans="1:7" ht="88" customHeight="1">
       <c r="A16" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>9</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="88" customHeight="1">
       <c r="A17" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>9</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="105.5" customHeight="1">
       <c r="A18" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>9</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="88" customHeight="1">
       <c r="A19" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="F19" s="1" t="s">
         <v>81</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="E19" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>86</v>
       </c>
       <c r="G19" s="1" t="s">
         <v>13</v>
@@ -1838,16 +1877,16 @@
   <sheetData>
     <row r="1" spans="1:6" ht="26.75" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>5</v>
@@ -1858,142 +1897,142 @@
     </row>
     <row r="2" spans="1:6" ht="70.25" customHeight="1">
       <c r="A2" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>104</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="47" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="70.25" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="70.25" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="70.25" customHeight="1">
       <c r="A6" s="1" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="70.25" customHeight="1">
       <c r="A7" s="1" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="70.25" customHeight="1">
       <c r="A8" s="1" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
     </row>
   </sheetData>
@@ -2015,7 +2054,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="26.75" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>3</v>
@@ -2032,138 +2071,138 @@
     </row>
     <row r="2" spans="1:5" ht="70.25" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="70.25" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="47" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="70.25" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="93.75" customHeight="1">
       <c r="A6" s="1" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="47" customHeight="1">
       <c r="A7" s="1" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="70.25" customHeight="1">
       <c r="A8" s="1" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="117.25" customHeight="1">
       <c r="A9" s="1" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
     </row>
   </sheetData>

</xml_diff>